<commit_message>
Correccion 02 - Baje soluciones para corregir
</commit_message>
<xml_diff>
--- a/Practicos/Archila Abel/Notas y devoluciones.xlsx
+++ b/Practicos/Archila Abel/Notas y devoluciones.xlsx
@@ -18,22 +18,38 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
-    <t>Nota:</t>
+    <t>Nota: 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+🎉¡Felicitaciones por la entrega del Desafío 01! 🎉
+Abel, quería felicitarte por el trabajo que realizaste. 
+Destaco la correcta estructura del documento HTML, genial que hayas declarado el lenguaje del documento en español, estos pequeños detalles van sumando a la legibilidad de la estructura.
+El trabajo no es una copia de lo solicitado pero  la lógica en el orden de aplicación de uso de etiquetas de encabezado (h1, h2, etc..) y el manejo de etiquetas para textos es correcto. 
+Genial que usas estilos en una hoja externa css, quedo muy bien ¡
+Observaciones a tu trabajo son:
+•	Falto usar la etiqueta strong en algún texto para darle énfasis de manera que los motores de búsqueda lo tomen en cuenta, por ejemplo podías enfatizar términos claves como “MERN” o “fullstack”.
+Excelente trabajo ¡
+Tu nota en el Desafío 01 es: 10
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota: </t>
   </si>
   <si>
     <t>Observaciones:</t>
   </si>
   <si>
-    <t xml:space="preserve">Nota: </t>
+    <t>Nota:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -42,10 +58,21 @@
     </font>
     <font>
       <b/>
+      <sz val="14.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font/>
+    <font>
+      <sz val="12.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -143,15 +170,17 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="top"/>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -160,9 +189,13 @@
     <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="11" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -408,23 +441,23 @@
       <c r="E3" s="5"/>
       <c r="F3" s="6"/>
     </row>
-    <row r="4" ht="15.75" customHeight="1">
+    <row r="4" ht="70.5" customHeight="1">
       <c r="A4" s="7"/>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" ht="15.75" customHeight="1">
+    <row r="5" ht="70.5" customHeight="1">
       <c r="A5" s="7"/>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" ht="15.75" customHeight="1">
+    <row r="6" ht="70.5" customHeight="1">
       <c r="A6" s="7"/>
       <c r="F6" s="8"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
+    <row r="7" ht="70.5" customHeight="1">
       <c r="A7" s="7"/>
       <c r="F7" s="8"/>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
+    <row r="8" ht="110.25" customHeight="1">
       <c r="A8" s="9"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -1455,8 +1488,8 @@
       <c r="F2" s="3"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
+      <c r="A3" s="13" t="s">
+        <v>3</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -2502,8 +2535,8 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1"/>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
+      <c r="A2" s="14" t="s">
+        <v>4</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2512,8 +2545,8 @@
       <c r="F2" s="3"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
+      <c r="A3" s="13" t="s">
+        <v>3</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>

</xml_diff>

<commit_message>
Correccion 03 - Llegue hasta Castillo Enrique que no aparece registrado en sistema
</commit_message>
<xml_diff>
--- a/Practicos/Archila Abel/Notas y devoluciones.xlsx
+++ b/Practicos/Archila Abel/Notas y devoluciones.xlsx
@@ -18,9 +18,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Nota: 10</t>
+  </si>
+  <si>
+    <t>Nota:</t>
+  </si>
+  <si>
+    <t>Nota: 9</t>
+  </si>
+  <si>
+    <t>Observaciones:</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -36,13 +45,16 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Nota: </t>
-  </si>
-  <si>
-    <t>Observaciones:</t>
-  </si>
-  <si>
-    <t>Nota:</t>
+    <t xml:space="preserve"> 
+🎉¡Felicitaciones por la entrega del Desafío 02! 🎉 
+Abel, excelente trabajo, el resultado es el que se solicitó en el enunciado. 
+La estructura HTML esta impecable, destaco la correcta implementación de contenedores semánticos como main, section, footer, etc. El manejo de listas, textos y títulos es correcto. 
+La manipulación de enlaces absolutos quedo perfecto. Genial que aplicaste pseudoclases para los enlaces.  
+La vinculación de la página de estilos externa es correcta, buenisimo que usaste id’s y clases , quedo genial. El diseño quedo distinto, pero se ve genial! 
+Destaco que completaste los atributos alt de las imágenes, esto ayuda a mejorar la accesibilidad de sito web.  
+Excelente trabajo ¡ 
+Tu nota en el Desafío 02 es: 9 
+</t>
   </si>
 </sst>
 </file>
@@ -62,14 +74,14 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
     <font/>
     <font>
       <sz val="12.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -170,32 +182,29 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="11" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="11" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -425,45 +434,45 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
+      <c r="A3" s="6" t="s">
+        <v>4</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
     </row>
     <row r="4" ht="70.5" customHeight="1">
-      <c r="A4" s="7"/>
-      <c r="F4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="F4" s="10"/>
     </row>
     <row r="5" ht="70.5" customHeight="1">
-      <c r="A5" s="7"/>
-      <c r="F5" s="8"/>
+      <c r="A5" s="9"/>
+      <c r="F5" s="10"/>
     </row>
     <row r="6" ht="70.5" customHeight="1">
-      <c r="A6" s="7"/>
-      <c r="F6" s="8"/>
+      <c r="A6" s="9"/>
+      <c r="F6" s="10"/>
     </row>
     <row r="7" ht="70.5" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="F7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="F7" s="10"/>
     </row>
     <row r="8" ht="110.25" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="13"/>
     </row>
     <row r="9" ht="15.75" customHeight="1"/>
     <row r="10" ht="15.75" customHeight="1"/>
@@ -1473,53 +1482,54 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="12.63"/>
+    <col customWidth="1" min="1" max="4" width="12.63"/>
+    <col customWidth="1" min="5" max="6" width="20.13"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1"/>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="13" t="s">
-        <v>3</v>
+      <c r="A3" s="6" t="s">
+        <v>5</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
     </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="7"/>
-      <c r="F4" s="8"/>
+    <row r="4" ht="70.5" customHeight="1">
+      <c r="A4" s="9"/>
+      <c r="F4" s="10"/>
     </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="7"/>
-      <c r="F5" s="8"/>
+    <row r="5" ht="70.5" customHeight="1">
+      <c r="A5" s="9"/>
+      <c r="F5" s="10"/>
     </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="7"/>
-      <c r="F6" s="8"/>
+    <row r="6" ht="70.5" customHeight="1">
+      <c r="A6" s="9"/>
+      <c r="F6" s="10"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="F7" s="8"/>
+    <row r="7" ht="142.5" customHeight="1">
+      <c r="A7" s="9"/>
+      <c r="F7" s="10"/>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11"/>
+    <row r="8" ht="142.5" customHeight="1">
+      <c r="A8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="13"/>
     </row>
     <row r="9" ht="15.75" customHeight="1"/>
     <row r="10" ht="15.75" customHeight="1"/>
@@ -2535,48 +2545,48 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1"/>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="14" t="s">
-        <v>4</v>
+      <c r="A2" s="2" t="s">
+        <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="7"/>
-      <c r="F4" s="8"/>
+      <c r="A4" s="9"/>
+      <c r="F4" s="10"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="7"/>
-      <c r="F5" s="8"/>
+      <c r="A5" s="9"/>
+      <c r="F5" s="10"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="7"/>
-      <c r="F6" s="8"/>
+      <c r="A6" s="9"/>
+      <c r="F6" s="10"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="F7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="F7" s="10"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="13"/>
     </row>
     <row r="9" ht="15.75" customHeight="1"/>
     <row r="10" ht="15.75" customHeight="1"/>

</xml_diff>